<commit_message>
feat: gestao de efetivo pelo administrador e login unificado por saram cpf e ldap comara.intraer
</commit_message>
<xml_diff>
--- a/data/efetivo_comara_oficial.xlsx
+++ b/data/efetivo_comara_oficial.xlsx
@@ -438,7 +438,7 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
@@ -539,7 +539,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>PRESIDENCIA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>PRESIDENCIA</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>PRESIDENCIA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -15140,7 +15140,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Claudio Valério Teles</t>
+          <t>Cláudio Valério Teles</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -15380,7 +15380,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>PRESIDENCIA</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">

</xml_diff>

<commit_message>
fix(fotos): correcao do mapeamento de saram no upload e integracao estrita com sigpesApi fotoes intraer
</commit_message>
<xml_diff>
--- a/data/efetivo_comara_oficial.xlsx
+++ b/data/efetivo_comara_oficial.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3800000</t>
+          <t>0804460</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3800001</t>
+          <t>2408589</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7000002</t>
+          <t>2282100</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3800003</t>
+          <t>0948292</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3800004</t>
+          <t>0010359</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3800005</t>
+          <t>3438708</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3800006</t>
+          <t>3100790</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3800007</t>
+          <t>3290972</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3800008</t>
+          <t>1741985</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>6000060</t>
+          <t>6032885</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>6000061</t>
+          <t>6088708</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>6000062</t>
+          <t>6210139</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>6000063</t>
+          <t>4199855</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>6000064</t>
+          <t>1676431</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>6000065</t>
+          <t>2991284</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>7000154</t>
+          <t>4388445</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -9006,7 +9006,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>7000155</t>
+          <t>4338790</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>7000156</t>
+          <t>4228812</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -9116,7 +9116,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>7000157</t>
+          <t>0917214</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">

</xml_diff>